<commit_message>
Add cost-to-shelf traceability slide and strip cost figures from shelf-price charts
- New slide 27 traces 105 and 122 UAH step by step from Self-Cost_Sias.xlsx
  (cost per unit, FX 51.20) through the partner-price formula to the shelf,
  and shows why the source workbook opens on a different cost row.
- Remove EUR cost-of-goods from the value column of the shelf-price bar
  charts: that column is UAH shelf price, and only our bars carried a second
  unit.
- Rename supply-volume labels and segment names in the workbook to the
  wording used in the supplier documents.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/Korean_Ramen_Model_and_Data.xlsx
+++ b/Korean_Ramen_Model_and_Data.xlsx
@@ -631,7 +631,7 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Тариф</t>
+          <t>Обсяг поставки</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D13" s="12" t="n">
@@ -740,7 +740,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D14" s="12" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
@@ -838,7 +838,7 @@
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D16" s="12" t="n">
@@ -887,7 +887,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D17" s="12" t="n">
@@ -936,7 +936,7 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="D18" s="12" t="n">
@@ -985,7 +985,7 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D19" s="12" t="n">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D20" s="12" t="n">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D21" s="12" t="n">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D23" s="12" t="n">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="D24" s="12" t="n">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D25" s="12" t="n">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D26" s="12" t="n">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D27" s="12" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D28" s="12" t="n">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D29" s="12" t="n">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="D30" s="12" t="n">
@@ -1592,12 +1592,12 @@
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>До €1,018 (стір-фрай)</t>
+          <t>До €1,018 (рамен із соусом)</t>
         </is>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
-          <t>До €0,882 (суповий)</t>
+          <t>До €0,882 (рамен з бульйоном)</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>Медіана сегмента 2 · стір-фрай</t>
+          <t>Медіана сегмента 2 · рамен із соусом</t>
         </is>
       </c>
       <c r="B36" s="21" t="n">
@@ -1682,7 +1682,7 @@
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>Медіана сегмента 1 · суповий</t>
+          <t>Медіана сегмента 1 · рамен з бульйоном</t>
         </is>
       </c>
       <c r="B37" s="21" t="n">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>Тариф</t>
+          <t>Обсяг поставки</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
@@ -1804,7 +1804,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Медіана сегмента 1 · суповий</t>
+          <t>Медіана сегмента 1 · рамен з бульйоном</t>
         </is>
       </c>
       <c r="B44" s="28" t="n">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="E44" s="13">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="E45" s="18">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="E46" s="13">
@@ -1889,7 +1889,7 @@
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>Медіана сегмента 2 · стір-фрай</t>
+          <t>Медіана сегмента 2 · рамен із соусом</t>
         </is>
       </c>
       <c r="B47" s="28" t="n">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="D47" s="17" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="E47" s="18">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="E48" s="13">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="D49" s="17" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="E49" s="18">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="E50" s="13">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="E51" s="18">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="E52" s="13">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="D53" s="17" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="E53" s="18">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="E54" s="13">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="D55" s="17" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="E55" s="18">
@@ -2151,7 +2151,7 @@
     <row r="59" ht="26" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Тариф</t>
+          <t>Обсяг поставки</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>6 палет</t>
+          <t>Мінімальний обсяг</t>
         </is>
       </c>
       <c r="B60" s="31" t="n">
@@ -2206,7 +2206,7 @@
     <row r="61">
       <c r="A61" s="17" t="inlineStr">
         <is>
-          <t>12 палет</t>
+          <t>Середній обсяг</t>
         </is>
       </c>
       <c r="B61" s="33" t="n">
@@ -2229,7 +2229,7 @@
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>33 палети</t>
+          <t>Максимальний обсяг</t>
         </is>
       </c>
       <c r="B62" s="31" t="n">
@@ -8221,17 +8221,17 @@
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>Ірландія</t>
+          <t>Японія</t>
         </is>
       </c>
       <c r="B26" s="33" t="n">
-        <v>45</v>
+        <v>192</v>
       </c>
       <c r="C26" s="33" t="n">
-        <v>386.41</v>
+        <v>1473.247</v>
       </c>
       <c r="D26" s="34" t="n">
-        <v>8.58688888888889</v>
+        <v>7.673161458333333</v>
       </c>
       <c r="E26" s="33" t="n"/>
       <c r="F26" s="33" t="n"/>
@@ -8241,17 +8241,17 @@
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
         <is>
-          <t>Японія</t>
+          <t>Ірландія</t>
         </is>
       </c>
       <c r="B27" s="31" t="n">
-        <v>192</v>
+        <v>45</v>
       </c>
       <c r="C27" s="31" t="n">
-        <v>1473.247</v>
+        <v>386.41</v>
       </c>
       <c r="D27" s="32" t="n">
-        <v>7.673161458333333</v>
+        <v>8.58688888888889</v>
       </c>
       <c r="E27" s="31" t="n"/>
       <c r="F27" s="31" t="n"/>

</xml_diff>